<commit_message>
PUG batch 1: verify buy links, write pillar copy, build import script
- Corrected Auntie Rana's (hummus -> Smoked Chili Oil, olive-oils category)
  and Felicia (legumes -> grains, pasta) after live-verification caught
  the original research miscategorizing both.
- Live-verified buy links + wrote 4-pillar copy for 12 approved brands:
  Brass Roots, Cactus Crunch, Chocxo, Dirtbag Bar, edggies veggies,
  Figa Foods, Figure Ate Foods (persimmon vinegar), Bake Away, DEFI Snacks,
  Auntie Rana's, Felicia, All The Bitter.
- Skipped Evo Hemp (signaled hemp protein bar line no longer sold on
  evohemp.com) and Brightland (duplicate of live Brightland Alive EVOO).
- scripts/import-pug-batch1.mjs ready to run against Airtable.
</commit_message>
<xml_diff>
--- a/global_brand_shortlist.xlsx
+++ b/global_brand_shortlist.xlsx
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1046,6 +1046,43 @@
       </c>
       <c r="G13" s="4" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Felicia (Andriani S.p.A.)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Organic buckwheat/whole-grain gluten-free pasta</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Parent company Andriani S.p.A. is a certified B Corp</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Felicia is the consumer brand of Andriani S.p.A. (already a verified B Corp in this shortlist's Grains sheet) -- vertically integrated supply chain of 500+ farmers across ~8,500 hectares, largest dried-legume supplier in Italy. Note: may overlap with the existing Andriani row -- confirm before adding both.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>https://felicia.us/about-felicia/</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1057,7 +1094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1402,72 +1439,6 @@
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Auntie Rana's</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Hummus</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>5% of profits donated to wildlife conservation</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Founder-driven, named percentage commitment (5% of profits) to protect endangered species (elephants, macaques, Irrawaddy dolphins) tied directly to her childhood in Bangladesh.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>https://auntieranas.com/</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Felicia (Andriani S.p.A.)</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Organic legume &amp; grain pasta (lentil, buckwheat, spirulina)</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Parent company Andriani S.p.A. is a certified B Corp</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Felicia is the consumer brand of Andriani S.p.A. (already a verified B Corp in this shortlist's Grains sheet) -- vertically integrated supply chain of 500+ farmers across ~8,500 hectares, largest dried-legume supplier in Italy. Note: may overlap with the existing Andriani row -- confirm before adding both.</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>https://felicia.us/about-felicia/</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1956,7 +1927,11 @@
           <t>https://brassrootsfood.com/</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1989,7 +1964,11 @@
           <t>https://cactus-foods.com/</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2022,7 +2001,11 @@
           <t>https://chocxo.com/pages/about-chocxo</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2055,7 +2038,11 @@
           <t>https://www.dirtbagbar.com/</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n"/>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2088,7 +2075,11 @@
           <t>https://www.edggies.com/pages/about</t>
         </is>
       </c>
-      <c r="G18" s="5" t="n"/>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2121,7 +2112,11 @@
           <t>https://evohemp.com/</t>
         </is>
       </c>
-      <c r="G19" s="5" t="n"/>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>N (bar line discontinued — see note)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2154,7 +2149,11 @@
           <t>https://figafoods.com/pages/about-us</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2187,7 +2186,11 @@
           <t>https://figureatefoods.com/</t>
         </is>
       </c>
-      <c r="G21" s="5" t="n"/>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Y (imported under Olive Oils &amp; Condiments as persimmon vinegar)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2220,7 +2223,11 @@
           <t>https://bakeaway.com/pages/about-us</t>
         </is>
       </c>
-      <c r="G22" s="5" t="n"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2253,7 +2260,11 @@
           <t>https://www.defisnacks.com/</t>
         </is>
       </c>
-      <c r="G23" s="5" t="n"/>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2775,7 +2786,11 @@
           <t>https://allthebitter.com/</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2788,7 +2803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2868,7 +2883,48 @@
           <t>https://brightland.co/pages/about-brightland-olive-oil</t>
         </is>
       </c>
-      <c r="G2" s="5" t="n"/>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>N (duplicate — already live as Brightland Alive EVOO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Auntie Rana's</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Smoked Chili Oil (condiment)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>5% of profits donated to wildlife conservation</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Founder-driven, named percentage commitment (5% of profits) to protect endangered species via partnerships with Wildlife SOS (India) and Wildlife Alliance (Cambodia), tied to founder's childhood in Bangladesh. Corrected from initial research: brand is a Southeast Asian condiments line (chili oil, mayo, achaar, jam), not a hummus/legumes product.</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>https://auntieranas.com/products/smoked-chili-oil</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Screen PUG batch 2 (25 brands): 7 shortlisted, 2 on hold, 15 rejected/duplicate
Shortlisted: Good Twin (LNA), Harken Sweets, Harry's Famous Sauce,
iMind Brain Food, Joey Nordic Seed Crisps, kencko, Kittylamb.
Hold pending direct verification: GOOD GREED, Kaizen Food Company.
Kahawa 1893 and MALK Organics rejected on category-fit grounds only
(coffee and oat milk don't map to any of the 6 GFA categories) despite
strong ethical signals -- flagged for Giovanni in case categories expand.
Kosterina rejected as duplicate of existing live product.
</commit_message>
<xml_diff>
--- a/global_brand_shortlist.xlsx
+++ b/global_brand_shortlist.xlsx
@@ -1451,7 +1451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2266,6 +2266,171 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Harken Sweets</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Plant-based, no-sugar-added candy bars</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Fair Trade certified</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Plant-based reimagining of classic candy bars (Snickers/Milky Way-style) with Fair Trade certified cocoa, 75% less sugar, 13g prebiotic fiber per bar.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>https://harkensweets.com/</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>iMind Brain Food</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Brain-health food bars</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Certified Organic (95%+ organic material)</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Founded by a board-certified neurosurgeon; bars blend organic whole-food ingredients and functional botanicals. Certified organic status verified via retail sustainability-feature badge, not just brand claim.</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.imindbrainfood.com/</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Joey Nordic Seed Crisps</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Canada (Prince Edward County)</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Seed crisps/crackers</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Certified organic, gluten-free</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Certified organic, gluten-free crisps made from 7 super seeds including upcycled watermelon seeds -- among the first snack brands to use upcycled watermelon seed as a protein source.</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>https://joeynordicseedcrisps.com/</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>kencko</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>USA / Portugal</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Organic instant smoothies, snacks</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Certified B Corp (92.0 score)</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Flash-frozen, slow-dried organic fruit and vegetable smoothie powders; Certified B Corporation with a B Impact score of 92.0, independently verified by B Lab. 100% organic, no added sugar.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/kencko/</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Kittylamb</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>USA (Scarborough, ME)</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Organic baking mixes</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>MOFGA certified organic</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Certified organic (MOFGA -- Maine Organic Farmers and Gardeners Association, an independent state-level certifier) baking mixes using fair-trade ingredients where available.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>https://kittylamb.com/</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2277,7 +2442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2792,6 +2957,39 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Good Twin</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>USA (Santa Maria, CA) / Italy-produced</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Non-alcoholic sparkling wine (Glera grape)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Certified organic (Bios Srl, Italian organic certifier)</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Made with real Glera grapes (the Prosecco variety), 4 ingredients, certified organic and vegan by Bios Srl -- an independent EU organic certification body, not a self-declared claim.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>https://drinkgoodtwin.com/</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2803,7 +3001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2926,6 +3124,39 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Harry's Famous Sauce</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Pasta sauces</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Non-GMO Project Verified + Upcycled Certified (select SKUs)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Founded by Harry Hamlin and Chef Renee Guilbault as debut line from The Open Food Company. Lemon Pepper Dill and Marinara No. 7 are Non-GMO Project certified; Lemon Pepper Dill is additionally Upcycled Certified via a Matriark Foods collaboration -- both independently audited certifications, not self-declared.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>https://harrysfamous.com/pages/about</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
PUG batch 2: verify buy links, write pillar copy, build import script
Live-verified buy links + wrote 4-pillar copy for 8 approved brands:
Good Twin, Harken Sweets, Harry's Famous Sauce, Joey Nordic Seed Crisps,
kencko, Kittylamb, Kahawa 1893 Coffee, MALK Organics.

Corrected two earlier category-fit rejections after closer look at
existing sheet precedent: Kahawa 1893 (coffee) fits Low & No Alcohol
same as existing yerba mate brands; MALK (oat milk) fits Snacks & Pantry
since it's shelf-stable, not perishable dairy like the earlier Boss Cow
rejection.

Skipped iMind Brain Food: out of stock everywhere checked (official site
+ 3 distinct Amazon ASINs, all unavailable).

scripts/import-pug-batch2.mjs ready to run against Airtable.
</commit_message>
<xml_diff>
--- a/global_brand_shortlist.xlsx
+++ b/global_brand_shortlist.xlsx
@@ -1451,7 +1451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2297,7 +2297,11 @@
           <t>https://harkensweets.com/</t>
         </is>
       </c>
-      <c r="G24" s="4" t="n"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2330,7 +2334,11 @@
           <t>https://www.imindbrainfood.com/</t>
         </is>
       </c>
-      <c r="G25" s="4" t="n"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>N (out of stock everywhere -- official site + 3 Amazon ASINs unavailable)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2363,7 +2371,11 @@
           <t>https://joeynordicseedcrisps.com/</t>
         </is>
       </c>
-      <c r="G26" s="4" t="n"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2396,7 +2408,11 @@
           <t>https://www.bcorporation.net/en-us/find-a-b-corp/company/kencko/</t>
         </is>
       </c>
-      <c r="G27" s="4" t="n"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2429,7 +2445,48 @@
           <t>https://kittylamb.com/</t>
         </is>
       </c>
-      <c r="G28" s="4" t="n"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>MALK Organics</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Shelf-stable oat/almond milk</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>USDA Organic</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>3-ingredient shelf-stable oat milk (filtered water, organic oats, Himalayan pink salt) -- USDA Organic certified, no gums/oils/fillers. Shelf-stable format distinguishes it from perishable refrigerated dairy alternatives.</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>https://malkorganics.com/products/oat-milk</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2442,7 +2499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2988,7 +3045,48 @@
           <t>https://drinkgoodtwin.com/</t>
         </is>
       </c>
-      <c r="G16" s="4" t="n"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Kahawa 1893 Coffee</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>USA / Kenya, Rwanda, Congo sourced</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Coffee (whole bean/ground)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Direct trade, women farmer-owned model</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Sources directly from women farmers in Kenya, Rwanda, and Congo, paying more than double the Fair Trade minimum price. Founder Margaret Nyamumbo pledges 25% of revenue to loans empowering women farmers, and the company matches customer tips to farmers dollar-for-dollar. First Black woman-owned coffee brand sold in Trader Joe's.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>https://kahawa1893.com/pages/fairtrade</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3155,7 +3253,11 @@
           <t>https://harrysfamous.com/pages/about</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>